<commit_message>
Simplify roles and add data import export
</commit_message>
<xml_diff>
--- a/data-templates/cpc1hn_data_import_template.xlsx
+++ b/data-templates/cpc1hn_data_import_template.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R329dee6ba92a489b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="Redd57f82c2d74fcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_dia_ban" sheetId="3" r:id="R87ad19695e844302"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_nhan_su" sheetId="4" r:id="R0bb1447e40184439"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="employee_territories" sheetId="5" r:id="Rad1df33de7a24932"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_san_pham" sheetId="6" r:id="R8bdc7431461a4c37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_khach_hang" sheetId="7" r:id="Rf1dfa58b594e49e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="employee_customers" sheetId="8" r:id="Rd4a74a03c2684e74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_ke_don" sheetId="9" r:id="Rf7c58d1e3f414648"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_doanh_thu" sheetId="10" r:id="Rbca788d2566f4c00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_thau" sheetId="11" r:id="R50b22e738fcc4665"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="daily_reports" sheetId="12" r:id="R16a4fd465e5c4ca8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kpi_targets" sheetId="13" r:id="Rc9915c09eef24551"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R702349bf0e4b4e1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="Ra8a9980f25aa4a4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_dia_ban" sheetId="3" r:id="Rc46cfa1521a04d76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_nhan_su" sheetId="4" r:id="R32b00fa03f5342c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="employee_territories" sheetId="5" r:id="R813b6c1bfbbd4ae7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_san_pham" sheetId="6" r:id="R1f01bc060d1d4ec8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_khach_hang" sheetId="7" r:id="R176d57c8645e4e23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="employee_customers" sheetId="8" r:id="Ref1860e2c1d045ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_ke_don" sheetId="9" r:id="R640e908dd1444364"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_doanh_thu" sheetId="10" r:id="R7355f15e03d4430f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_thau" sheetId="11" r:id="R95f7c279f00042c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="daily_reports" sheetId="12" r:id="R96020635f0394c03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kpi_targets" sheetId="13" r:id="R2168ac9e86b94d89"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2541,7 +2541,7 @@
   <x:cols>
     <x:col min="1" max="1" width="24.8799991607666" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="13.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="17.8799991607666" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="47" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -2565,10 +2565,10 @@
         <x:v>chuc_vu</x:v>
       </x:c>
       <x:c r="B4" s="3" t="str">
-        <x:v>MR</x:v>
+        <x:v>NhanVien</x:v>
       </x:c>
       <x:c r="C4" s="3" t="str">
-        <x:v>Trình dược viên</x:v>
+        <x:v>Nhân viên nhập dữ liệu theo khách hàng được phân công</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -2576,54 +2576,54 @@
         <x:v>chuc_vu</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>Supervisor</x:v>
+        <x:v>QuanLy</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
-        <x:v>Quản lý vùng</x:v>
+        <x:v>Quản lý toàn hệ thống, được quản trị và import/export dữ liệu</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="3" t="str">
-        <x:v>chuc_vu</x:v>
+        <x:v>trang_thai</x:v>
       </x:c>
       <x:c r="B6" s="3" t="str">
-        <x:v>Manager</x:v>
+        <x:v>Active</x:v>
       </x:c>
       <x:c r="C6" s="3" t="str">
-        <x:v>Quản lý toàn hệ thống</x:v>
+        <x:v>Đang hoạt động</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="3" t="str">
-        <x:v>chuc_vu</x:v>
+        <x:v>trang_thai</x:v>
       </x:c>
       <x:c r="B7" s="3" t="str">
-        <x:v>Admin</x:v>
+        <x:v>Inactive</x:v>
       </x:c>
       <x:c r="C7" s="3" t="str">
-        <x:v>Quản trị hệ thống</x:v>
+        <x:v>Ngừng hoạt động</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="3" t="str">
-        <x:v>trang_thai</x:v>
+        <x:v>loai_khach_hang</x:v>
       </x:c>
       <x:c r="B8" s="3" t="str">
-        <x:v>Active</x:v>
+        <x:v>BenhVien</x:v>
       </x:c>
       <x:c r="C8" s="3" t="str">
-        <x:v>Đang hoạt động</x:v>
+        <x:v>Bệnh viện</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="3" t="str">
-        <x:v>trang_thai</x:v>
+        <x:v>loai_khach_hang</x:v>
       </x:c>
       <x:c r="B9" s="3" t="str">
-        <x:v>Inactive</x:v>
+        <x:v>SoYTe</x:v>
       </x:c>
       <x:c r="C9" s="3" t="str">
-        <x:v>Ngừng hoạt động</x:v>
+        <x:v>Sở Y tế</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2631,32 +2631,32 @@
         <x:v>loai_khach_hang</x:v>
       </x:c>
       <x:c r="B10" s="3" t="str">
-        <x:v>BenhVien</x:v>
+        <x:v>PhongMachTu</x:v>
       </x:c>
       <x:c r="C10" s="3" t="str">
-        <x:v>Bệnh viện</x:v>
+        <x:v>Phòng mạch tư nhân</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="3" t="str">
-        <x:v>loai_khach_hang</x:v>
+        <x:v>dang_bao_che</x:v>
       </x:c>
       <x:c r="B11" s="3" t="str">
-        <x:v>SoYTe</x:v>
+        <x:v>BFS</x:v>
       </x:c>
       <x:c r="C11" s="3" t="str">
-        <x:v>Sở Y tế</x:v>
+        <x:v>Dung dịch khí dung BFS</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="3" t="str">
-        <x:v>loai_khach_hang</x:v>
+        <x:v>dang_bao_che</x:v>
       </x:c>
       <x:c r="B12" s="3" t="str">
-        <x:v>PhongMachTu</x:v>
+        <x:v>BOV</x:v>
       </x:c>
       <x:c r="C12" s="3" t="str">
-        <x:v>Phòng mạch tư nhân</x:v>
+        <x:v>Bình xịt mũi BOV</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2664,10 +2664,10 @@
         <x:v>dang_bao_che</x:v>
       </x:c>
       <x:c r="B13" s="3" t="str">
-        <x:v>BFS</x:v>
+        <x:v>MDI</x:v>
       </x:c>
       <x:c r="C13" s="3" t="str">
-        <x:v>Dung dịch khí dung BFS</x:v>
+        <x:v>Ống hít định liều MDI</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2675,32 +2675,32 @@
         <x:v>dang_bao_che</x:v>
       </x:c>
       <x:c r="B14" s="3" t="str">
-        <x:v>BOV</x:v>
+        <x:v>VienDatDoKhuon</x:v>
       </x:c>
       <x:c r="C14" s="3" t="str">
-        <x:v>Bình xịt mũi BOV</x:v>
+        <x:v>Viên đặt đổ khuôn</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="3" t="str">
-        <x:v>dang_bao_che</x:v>
+        <x:v>trang_thai_thau</x:v>
       </x:c>
       <x:c r="B15" s="3" t="str">
-        <x:v>MDI</x:v>
+        <x:v>DangLamHoSo</x:v>
       </x:c>
       <x:c r="C15" s="3" t="str">
-        <x:v>Ống hít định liều MDI</x:v>
+        <x:v>Đang làm hồ sơ</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="3" t="str">
-        <x:v>dang_bao_che</x:v>
+        <x:v>trang_thai_thau</x:v>
       </x:c>
       <x:c r="B16" s="3" t="str">
-        <x:v>VienDatDoKhuon</x:v>
+        <x:v>ChoKetQua</x:v>
       </x:c>
       <x:c r="C16" s="3" t="str">
-        <x:v>Viên đặt đổ khuôn</x:v>
+        <x:v>Chờ kết quả</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2708,10 +2708,10 @@
         <x:v>trang_thai_thau</x:v>
       </x:c>
       <x:c r="B17" s="3" t="str">
-        <x:v>DangLamHoSo</x:v>
+        <x:v>TrungThau</x:v>
       </x:c>
       <x:c r="C17" s="3" t="str">
-        <x:v>Đang làm hồ sơ</x:v>
+        <x:v>Trúng thầu</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2719,31 +2719,9 @@
         <x:v>trang_thai_thau</x:v>
       </x:c>
       <x:c r="B18" s="3" t="str">
-        <x:v>ChoKetQua</x:v>
+        <x:v>TruotThau</x:v>
       </x:c>
       <x:c r="C18" s="3" t="str">
-        <x:v>Chờ kết quả</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="3" t="str">
-        <x:v>trang_thai_thau</x:v>
-      </x:c>
-      <x:c r="B19" s="3" t="str">
-        <x:v>TrungThau</x:v>
-      </x:c>
-      <x:c r="C19" s="3" t="str">
-        <x:v>Trúng thầu</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="3" t="str">
-        <x:v>trang_thai_thau</x:v>
-      </x:c>
-      <x:c r="B20" s="3" t="str">
-        <x:v>TruotThau</x:v>
-      </x:c>
-      <x:c r="C20" s="3" t="str">
         <x:v>Trượt thầu</x:v>
       </x:c>
     </x:row>
@@ -3067,10 +3045,10 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="68" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="57.130001068115234" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="19.8799991607666" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="10.5" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22.6299991607666" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="9.880000114440918" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="8.5" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -3081,7 +3059,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="14" t="str">
-        <x:v>Email phải đúng email đăng nhập. chuc_vu chỉ dùng MR, Supervisor, Manager hoặc Admin.</x:v>
+        <x:v>Email phải đúng email đăng nhập. chuc_vu chỉ dùng NhanVien hoặc QuanLy.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -3126,10 +3104,10 @@
         <x:v>Nguyễn Minh Anh</x:v>
       </x:c>
       <x:c r="C6" s="22" t="str">
-        <x:v>mr.danang@cpc1hn.vn</x:v>
+        <x:v>nhanvien.danang@cpc1hn.vn</x:v>
       </x:c>
       <x:c r="D6" s="21" t="str">
-        <x:v>MR</x:v>
+        <x:v>NhanVien</x:v>
       </x:c>
       <x:c r="E6" s="21" t="str">
         <x:v>Active</x:v>
@@ -3137,16 +3115,16 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="22" t="str">
-        <x:v>NV-SV-01</x:v>
+        <x:v>NV-QL-01</x:v>
       </x:c>
       <x:c r="B7" s="21" t="str">
-        <x:v>Lê Thu Hà</x:v>
+        <x:v>Phạm Quốc Bảo</x:v>
       </x:c>
       <x:c r="C7" s="22" t="str">
-        <x:v>supervisor.mt@cpc1hn.vn</x:v>
+        <x:v>quanly@cpc1hn.vn</x:v>
       </x:c>
       <x:c r="D7" s="21" t="str">
-        <x:v>Supervisor</x:v>
+        <x:v>QuanLy</x:v>
       </x:c>
       <x:c r="E7" s="21" t="str">
         <x:v>Active</x:v>
@@ -3481,7 +3459,7 @@
   </x:mergeCells>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="D6:D50">
-      <x:formula1>"MR,Supervisor,Manager,Admin"</x:formula1>
+      <x:formula1>"NhanVien,QuanLy"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="E6:E50">
       <x:formula1>"Active,Inactive"</x:formula1>
@@ -3545,7 +3523,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="22" t="str">
-        <x:v>NV-SV-01</x:v>
+        <x:v>NV-QL-01</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
         <x:v>DB_DANANG</x:v>
@@ -3556,7 +3534,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="22" t="str">
-        <x:v>NV-SV-01</x:v>
+        <x:v>NV-QL-01</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
         <x:v>DB_QUANGNAM</x:v>

</xml_diff>

<commit_message>
Migrate backend to Postgres and add DATA SALE import
</commit_message>
<xml_diff>
--- a/data-templates/cpc1hn_data_import_template.xlsx
+++ b/data-templates/cpc1hn_data_import_template.xlsx
@@ -2,19 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R702349bf0e4b4e1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="Ra8a9980f25aa4a4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_dia_ban" sheetId="3" r:id="Rc46cfa1521a04d76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_nhan_su" sheetId="4" r:id="R32b00fa03f5342c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="employee_territories" sheetId="5" r:id="R813b6c1bfbbd4ae7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_san_pham" sheetId="6" r:id="R1f01bc060d1d4ec8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_khach_hang" sheetId="7" r:id="R176d57c8645e4e23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="employee_customers" sheetId="8" r:id="Ref1860e2c1d045ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_ke_don" sheetId="9" r:id="R640e908dd1444364"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_doanh_thu" sheetId="10" r:id="R7355f15e03d4430f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_thau" sheetId="11" r:id="R95f7c279f00042c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="daily_reports" sheetId="12" r:id="R96020635f0394c03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kpi_targets" sheetId="13" r:id="R2168ac9e86b94d89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R05fcac19caec49d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="R1661de6de30f444a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_dia_ban" sheetId="3" r:id="R24d53b6af0234ede"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_nhan_su" sheetId="4" r:id="Raa7ed7f14d6e4ed9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="employee_territories" sheetId="5" r:id="R3faf448cf2914b3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_san_pham" sheetId="6" r:id="Rbcf15486bb814392"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_khach_hang" sheetId="7" r:id="R5343503bfe31476e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="employee_customers" sheetId="8" r:id="R3b54975bdc344552"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_ke_don" sheetId="9" r:id="Rcbbf3cb652944185"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_doanh_thu" sheetId="10" r:id="R023c1a70756b4db4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_sale_transactions" sheetId="11" r:id="R620cf4dcc265470e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tb_thau" sheetId="12" r:id="R86179e8d8bf7498f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="daily_reports" sheetId="13" r:id="Rb04c25123ebe4dfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kpi_targets" sheetId="14" r:id="Rf872052ed67f4a4c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,10 +26,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
     <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="203" formatCode="#,##0.###"/>
+    <x:numFmt numFmtId="204" formatCode="#,##0.000"/>
+    <x:numFmt numFmtId="205" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="206" formatCode="0.####"/>
   </x:numFmts>
   <x:fonts count="7">
     <x:font>
@@ -121,7 +126,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="35">
+  <x:cellXfs count="39">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -218,6 +223,18 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="202" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1055,14 +1072,1222 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="9" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="34" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="13" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="36" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="10" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="14" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="16" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="11" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="16" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="2" t="str">
+        <x:v>DATA SALE chi tiết</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="14" t="str">
+        <x:v>Giữ nguyên 19 cột A:S từ Google Sheet DATA SALE. Mã nhân viên phải là text để giữ số 0 đầu. Ngày xuất CSV nên chuẩn hóa yyyy-mm-dd.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="6" t="str">
+        <x:v>Quản lý</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="str">
+        <x:v>NV kinh doanh</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="str">
+        <x:v>Tên NV KD</x:v>
+      </x:c>
+      <x:c r="D4" s="6" t="str">
+        <x:v>Tỉnh</x:v>
+      </x:c>
+      <x:c r="E4" s="6" t="str">
+        <x:v>Nhóm KH</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="str">
+        <x:v>Tháng</x:v>
+      </x:c>
+      <x:c r="G4" s="6" t="str">
+        <x:v>Năm</x:v>
+      </x:c>
+      <x:c r="H4" s="6" t="str">
+        <x:v>Mã Kh</x:v>
+      </x:c>
+      <x:c r="I4" s="6" t="str">
+        <x:v>Tên KH</x:v>
+      </x:c>
+      <x:c r="J4" s="6" t="str">
+        <x:v>Ngày chứng từ</x:v>
+      </x:c>
+      <x:c r="K4" s="6" t="str">
+        <x:v>Số Chứng từ ngoại</x:v>
+      </x:c>
+      <x:c r="L4" s="6" t="str">
+        <x:v>Mã HH</x:v>
+      </x:c>
+      <x:c r="M4" s="6" t="str">
+        <x:v>Tên HH</x:v>
+      </x:c>
+      <x:c r="N4" s="6" t="str">
+        <x:v>DVT</x:v>
+      </x:c>
+      <x:c r="O4" s="6" t="str">
+        <x:v>Số Lượng</x:v>
+      </x:c>
+      <x:c r="P4" s="6" t="str">
+        <x:v>Đơn giá</x:v>
+      </x:c>
+      <x:c r="Q4" s="6" t="str">
+        <x:v>Doanh thu</x:v>
+      </x:c>
+      <x:c r="R4" s="6" t="str">
+        <x:v>Hệ số</x:v>
+      </x:c>
+      <x:c r="S4" s="6" t="str">
+        <x:v>DOANH SỐ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="18" t="str">
+        <x:v>Không bắt buộc</x:v>
+      </x:c>
+      <x:c r="B5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="C5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="D5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="E5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="F5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="G5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="H5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="I5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="J5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="K5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="L5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="M5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="N5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="O5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="P5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="Q5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="R5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+      <x:c r="S5" s="18" t="str">
+        <x:v>Bắt buộc</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="29" t="str">
+        <x:v>Trương Anh Tú</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>015795</x:v>
+      </x:c>
+      <x:c r="C6" s="21" t="str">
+        <x:v>Nguyễn Ngọc Phương Thảo</x:v>
+      </x:c>
+      <x:c r="D6" s="21" t="str">
+        <x:v>Quảng Nam</x:v>
+      </x:c>
+      <x:c r="E6" s="21" t="str">
+        <x:v>BV Kê đơn</x:v>
+      </x:c>
+      <x:c r="F6" s="21" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G6" s="21" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="H6" s="22" t="str">
+        <x:v>KC01287</x:v>
+      </x:c>
+      <x:c r="I6" s="21" t="str">
+        <x:v>Công Ty TNHH Y Khoa Minh Trí Hội An</x:v>
+      </x:c>
+      <x:c r="J6" s="31" t="n">
+        <x:v>45659</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="str">
+        <x:v>FB2531/00025</x:v>
+      </x:c>
+      <x:c r="L6" s="22" t="str">
+        <x:v>W00504</x:v>
+      </x:c>
+      <x:c r="M6" s="21" t="str">
+        <x:v>Hylaform 0,1% 10ml</x:v>
+      </x:c>
+      <x:c r="N6" s="21" t="str">
+        <x:v>ONG</x:v>
+      </x:c>
+      <x:c r="O6" s="33" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="P6" s="34" t="n">
+        <x:v>30714.286</x:v>
+      </x:c>
+      <x:c r="Q6" s="35" t="n">
+        <x:v>1228571</x:v>
+      </x:c>
+      <x:c r="R6" s="36" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="S6" s="35" t="n">
+        <x:v>1842856.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="29"/>
+      <x:c r="B7" s="22"/>
+      <x:c r="C7" s="21"/>
+      <x:c r="D7" s="21"/>
+      <x:c r="E7" s="21"/>
+      <x:c r="F7" s="21"/>
+      <x:c r="G7" s="21"/>
+      <x:c r="H7" s="22"/>
+      <x:c r="I7" s="21"/>
+      <x:c r="J7" s="31"/>
+      <x:c r="K7" s="22"/>
+      <x:c r="L7" s="22"/>
+      <x:c r="M7" s="21"/>
+      <x:c r="N7" s="21"/>
+      <x:c r="O7" s="33"/>
+      <x:c r="P7" s="34"/>
+      <x:c r="Q7" s="35"/>
+      <x:c r="R7" s="36"/>
+      <x:c r="S7" s="35"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="29"/>
+      <x:c r="B8" s="22"/>
+      <x:c r="C8" s="21"/>
+      <x:c r="D8" s="21"/>
+      <x:c r="E8" s="21"/>
+      <x:c r="F8" s="21"/>
+      <x:c r="G8" s="21"/>
+      <x:c r="H8" s="22"/>
+      <x:c r="I8" s="21"/>
+      <x:c r="J8" s="31"/>
+      <x:c r="K8" s="22"/>
+      <x:c r="L8" s="22"/>
+      <x:c r="M8" s="21"/>
+      <x:c r="N8" s="21"/>
+      <x:c r="O8" s="33"/>
+      <x:c r="P8" s="34"/>
+      <x:c r="Q8" s="35"/>
+      <x:c r="R8" s="36"/>
+      <x:c r="S8" s="35"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29"/>
+      <x:c r="B9" s="22"/>
+      <x:c r="C9" s="21"/>
+      <x:c r="D9" s="21"/>
+      <x:c r="E9" s="21"/>
+      <x:c r="F9" s="21"/>
+      <x:c r="G9" s="21"/>
+      <x:c r="H9" s="22"/>
+      <x:c r="I9" s="21"/>
+      <x:c r="J9" s="31"/>
+      <x:c r="K9" s="22"/>
+      <x:c r="L9" s="22"/>
+      <x:c r="M9" s="21"/>
+      <x:c r="N9" s="21"/>
+      <x:c r="O9" s="33"/>
+      <x:c r="P9" s="34"/>
+      <x:c r="Q9" s="35"/>
+      <x:c r="R9" s="36"/>
+      <x:c r="S9" s="35"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29"/>
+      <x:c r="B10" s="22"/>
+      <x:c r="C10" s="21"/>
+      <x:c r="D10" s="21"/>
+      <x:c r="E10" s="21"/>
+      <x:c r="F10" s="21"/>
+      <x:c r="G10" s="21"/>
+      <x:c r="H10" s="22"/>
+      <x:c r="I10" s="21"/>
+      <x:c r="J10" s="31"/>
+      <x:c r="K10" s="22"/>
+      <x:c r="L10" s="22"/>
+      <x:c r="M10" s="21"/>
+      <x:c r="N10" s="21"/>
+      <x:c r="O10" s="33"/>
+      <x:c r="P10" s="34"/>
+      <x:c r="Q10" s="35"/>
+      <x:c r="R10" s="36"/>
+      <x:c r="S10" s="35"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29"/>
+      <x:c r="B11" s="22"/>
+      <x:c r="C11" s="21"/>
+      <x:c r="D11" s="21"/>
+      <x:c r="E11" s="21"/>
+      <x:c r="F11" s="21"/>
+      <x:c r="G11" s="21"/>
+      <x:c r="H11" s="22"/>
+      <x:c r="I11" s="21"/>
+      <x:c r="J11" s="31"/>
+      <x:c r="K11" s="22"/>
+      <x:c r="L11" s="22"/>
+      <x:c r="M11" s="21"/>
+      <x:c r="N11" s="21"/>
+      <x:c r="O11" s="33"/>
+      <x:c r="P11" s="34"/>
+      <x:c r="Q11" s="35"/>
+      <x:c r="R11" s="36"/>
+      <x:c r="S11" s="35"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29"/>
+      <x:c r="B12" s="22"/>
+      <x:c r="C12" s="21"/>
+      <x:c r="D12" s="21"/>
+      <x:c r="E12" s="21"/>
+      <x:c r="F12" s="21"/>
+      <x:c r="G12" s="21"/>
+      <x:c r="H12" s="22"/>
+      <x:c r="I12" s="21"/>
+      <x:c r="J12" s="31"/>
+      <x:c r="K12" s="22"/>
+      <x:c r="L12" s="22"/>
+      <x:c r="M12" s="21"/>
+      <x:c r="N12" s="21"/>
+      <x:c r="O12" s="33"/>
+      <x:c r="P12" s="34"/>
+      <x:c r="Q12" s="35"/>
+      <x:c r="R12" s="36"/>
+      <x:c r="S12" s="35"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="29"/>
+      <x:c r="B13" s="22"/>
+      <x:c r="C13" s="21"/>
+      <x:c r="D13" s="21"/>
+      <x:c r="E13" s="21"/>
+      <x:c r="F13" s="21"/>
+      <x:c r="G13" s="21"/>
+      <x:c r="H13" s="22"/>
+      <x:c r="I13" s="21"/>
+      <x:c r="J13" s="31"/>
+      <x:c r="K13" s="22"/>
+      <x:c r="L13" s="22"/>
+      <x:c r="M13" s="21"/>
+      <x:c r="N13" s="21"/>
+      <x:c r="O13" s="33"/>
+      <x:c r="P13" s="34"/>
+      <x:c r="Q13" s="35"/>
+      <x:c r="R13" s="36"/>
+      <x:c r="S13" s="35"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29"/>
+      <x:c r="B14" s="22"/>
+      <x:c r="C14" s="21"/>
+      <x:c r="D14" s="21"/>
+      <x:c r="E14" s="21"/>
+      <x:c r="F14" s="21"/>
+      <x:c r="G14" s="21"/>
+      <x:c r="H14" s="22"/>
+      <x:c r="I14" s="21"/>
+      <x:c r="J14" s="31"/>
+      <x:c r="K14" s="22"/>
+      <x:c r="L14" s="22"/>
+      <x:c r="M14" s="21"/>
+      <x:c r="N14" s="21"/>
+      <x:c r="O14" s="33"/>
+      <x:c r="P14" s="34"/>
+      <x:c r="Q14" s="35"/>
+      <x:c r="R14" s="36"/>
+      <x:c r="S14" s="35"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="29"/>
+      <x:c r="B15" s="22"/>
+      <x:c r="C15" s="21"/>
+      <x:c r="D15" s="21"/>
+      <x:c r="E15" s="21"/>
+      <x:c r="F15" s="21"/>
+      <x:c r="G15" s="21"/>
+      <x:c r="H15" s="22"/>
+      <x:c r="I15" s="21"/>
+      <x:c r="J15" s="31"/>
+      <x:c r="K15" s="22"/>
+      <x:c r="L15" s="22"/>
+      <x:c r="M15" s="21"/>
+      <x:c r="N15" s="21"/>
+      <x:c r="O15" s="33"/>
+      <x:c r="P15" s="34"/>
+      <x:c r="Q15" s="35"/>
+      <x:c r="R15" s="36"/>
+      <x:c r="S15" s="35"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29"/>
+      <x:c r="B16" s="22"/>
+      <x:c r="C16" s="21"/>
+      <x:c r="D16" s="21"/>
+      <x:c r="E16" s="21"/>
+      <x:c r="F16" s="21"/>
+      <x:c r="G16" s="21"/>
+      <x:c r="H16" s="22"/>
+      <x:c r="I16" s="21"/>
+      <x:c r="J16" s="31"/>
+      <x:c r="K16" s="22"/>
+      <x:c r="L16" s="22"/>
+      <x:c r="M16" s="21"/>
+      <x:c r="N16" s="21"/>
+      <x:c r="O16" s="33"/>
+      <x:c r="P16" s="34"/>
+      <x:c r="Q16" s="35"/>
+      <x:c r="R16" s="36"/>
+      <x:c r="S16" s="35"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="29"/>
+      <x:c r="B17" s="22"/>
+      <x:c r="C17" s="21"/>
+      <x:c r="D17" s="21"/>
+      <x:c r="E17" s="21"/>
+      <x:c r="F17" s="21"/>
+      <x:c r="G17" s="21"/>
+      <x:c r="H17" s="22"/>
+      <x:c r="I17" s="21"/>
+      <x:c r="J17" s="31"/>
+      <x:c r="K17" s="22"/>
+      <x:c r="L17" s="22"/>
+      <x:c r="M17" s="21"/>
+      <x:c r="N17" s="21"/>
+      <x:c r="O17" s="33"/>
+      <x:c r="P17" s="34"/>
+      <x:c r="Q17" s="35"/>
+      <x:c r="R17" s="36"/>
+      <x:c r="S17" s="35"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="29"/>
+      <x:c r="B18" s="22"/>
+      <x:c r="C18" s="21"/>
+      <x:c r="D18" s="21"/>
+      <x:c r="E18" s="21"/>
+      <x:c r="F18" s="21"/>
+      <x:c r="G18" s="21"/>
+      <x:c r="H18" s="22"/>
+      <x:c r="I18" s="21"/>
+      <x:c r="J18" s="31"/>
+      <x:c r="K18" s="22"/>
+      <x:c r="L18" s="22"/>
+      <x:c r="M18" s="21"/>
+      <x:c r="N18" s="21"/>
+      <x:c r="O18" s="33"/>
+      <x:c r="P18" s="34"/>
+      <x:c r="Q18" s="35"/>
+      <x:c r="R18" s="36"/>
+      <x:c r="S18" s="35"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="29"/>
+      <x:c r="B19" s="22"/>
+      <x:c r="C19" s="21"/>
+      <x:c r="D19" s="21"/>
+      <x:c r="E19" s="21"/>
+      <x:c r="F19" s="21"/>
+      <x:c r="G19" s="21"/>
+      <x:c r="H19" s="22"/>
+      <x:c r="I19" s="21"/>
+      <x:c r="J19" s="31"/>
+      <x:c r="K19" s="22"/>
+      <x:c r="L19" s="22"/>
+      <x:c r="M19" s="21"/>
+      <x:c r="N19" s="21"/>
+      <x:c r="O19" s="33"/>
+      <x:c r="P19" s="34"/>
+      <x:c r="Q19" s="35"/>
+      <x:c r="R19" s="36"/>
+      <x:c r="S19" s="35"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="29"/>
+      <x:c r="B20" s="22"/>
+      <x:c r="C20" s="21"/>
+      <x:c r="D20" s="21"/>
+      <x:c r="E20" s="21"/>
+      <x:c r="F20" s="21"/>
+      <x:c r="G20" s="21"/>
+      <x:c r="H20" s="22"/>
+      <x:c r="I20" s="21"/>
+      <x:c r="J20" s="31"/>
+      <x:c r="K20" s="22"/>
+      <x:c r="L20" s="22"/>
+      <x:c r="M20" s="21"/>
+      <x:c r="N20" s="21"/>
+      <x:c r="O20" s="33"/>
+      <x:c r="P20" s="34"/>
+      <x:c r="Q20" s="35"/>
+      <x:c r="R20" s="36"/>
+      <x:c r="S20" s="35"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="29"/>
+      <x:c r="B21" s="22"/>
+      <x:c r="C21" s="21"/>
+      <x:c r="D21" s="21"/>
+      <x:c r="E21" s="21"/>
+      <x:c r="F21" s="21"/>
+      <x:c r="G21" s="21"/>
+      <x:c r="H21" s="22"/>
+      <x:c r="I21" s="21"/>
+      <x:c r="J21" s="31"/>
+      <x:c r="K21" s="22"/>
+      <x:c r="L21" s="22"/>
+      <x:c r="M21" s="21"/>
+      <x:c r="N21" s="21"/>
+      <x:c r="O21" s="33"/>
+      <x:c r="P21" s="34"/>
+      <x:c r="Q21" s="35"/>
+      <x:c r="R21" s="36"/>
+      <x:c r="S21" s="35"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="29"/>
+      <x:c r="B22" s="22"/>
+      <x:c r="C22" s="21"/>
+      <x:c r="D22" s="21"/>
+      <x:c r="E22" s="21"/>
+      <x:c r="F22" s="21"/>
+      <x:c r="G22" s="21"/>
+      <x:c r="H22" s="22"/>
+      <x:c r="I22" s="21"/>
+      <x:c r="J22" s="31"/>
+      <x:c r="K22" s="22"/>
+      <x:c r="L22" s="22"/>
+      <x:c r="M22" s="21"/>
+      <x:c r="N22" s="21"/>
+      <x:c r="O22" s="33"/>
+      <x:c r="P22" s="34"/>
+      <x:c r="Q22" s="35"/>
+      <x:c r="R22" s="36"/>
+      <x:c r="S22" s="35"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="29"/>
+      <x:c r="B23" s="22"/>
+      <x:c r="C23" s="21"/>
+      <x:c r="D23" s="21"/>
+      <x:c r="E23" s="21"/>
+      <x:c r="F23" s="21"/>
+      <x:c r="G23" s="21"/>
+      <x:c r="H23" s="22"/>
+      <x:c r="I23" s="21"/>
+      <x:c r="J23" s="31"/>
+      <x:c r="K23" s="22"/>
+      <x:c r="L23" s="22"/>
+      <x:c r="M23" s="21"/>
+      <x:c r="N23" s="21"/>
+      <x:c r="O23" s="33"/>
+      <x:c r="P23" s="34"/>
+      <x:c r="Q23" s="35"/>
+      <x:c r="R23" s="36"/>
+      <x:c r="S23" s="35"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="29"/>
+      <x:c r="B24" s="22"/>
+      <x:c r="C24" s="21"/>
+      <x:c r="D24" s="21"/>
+      <x:c r="E24" s="21"/>
+      <x:c r="F24" s="21"/>
+      <x:c r="G24" s="21"/>
+      <x:c r="H24" s="22"/>
+      <x:c r="I24" s="21"/>
+      <x:c r="J24" s="31"/>
+      <x:c r="K24" s="22"/>
+      <x:c r="L24" s="22"/>
+      <x:c r="M24" s="21"/>
+      <x:c r="N24" s="21"/>
+      <x:c r="O24" s="33"/>
+      <x:c r="P24" s="34"/>
+      <x:c r="Q24" s="35"/>
+      <x:c r="R24" s="36"/>
+      <x:c r="S24" s="35"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="29"/>
+      <x:c r="B25" s="22"/>
+      <x:c r="C25" s="21"/>
+      <x:c r="D25" s="21"/>
+      <x:c r="E25" s="21"/>
+      <x:c r="F25" s="21"/>
+      <x:c r="G25" s="21"/>
+      <x:c r="H25" s="22"/>
+      <x:c r="I25" s="21"/>
+      <x:c r="J25" s="31"/>
+      <x:c r="K25" s="22"/>
+      <x:c r="L25" s="22"/>
+      <x:c r="M25" s="21"/>
+      <x:c r="N25" s="21"/>
+      <x:c r="O25" s="33"/>
+      <x:c r="P25" s="34"/>
+      <x:c r="Q25" s="35"/>
+      <x:c r="R25" s="36"/>
+      <x:c r="S25" s="35"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="29"/>
+      <x:c r="B26" s="22"/>
+      <x:c r="C26" s="21"/>
+      <x:c r="D26" s="21"/>
+      <x:c r="E26" s="21"/>
+      <x:c r="F26" s="21"/>
+      <x:c r="G26" s="21"/>
+      <x:c r="H26" s="22"/>
+      <x:c r="I26" s="21"/>
+      <x:c r="J26" s="31"/>
+      <x:c r="K26" s="22"/>
+      <x:c r="L26" s="22"/>
+      <x:c r="M26" s="21"/>
+      <x:c r="N26" s="21"/>
+      <x:c r="O26" s="33"/>
+      <x:c r="P26" s="34"/>
+      <x:c r="Q26" s="35"/>
+      <x:c r="R26" s="36"/>
+      <x:c r="S26" s="35"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="29"/>
+      <x:c r="B27" s="22"/>
+      <x:c r="C27" s="21"/>
+      <x:c r="D27" s="21"/>
+      <x:c r="E27" s="21"/>
+      <x:c r="F27" s="21"/>
+      <x:c r="G27" s="21"/>
+      <x:c r="H27" s="22"/>
+      <x:c r="I27" s="21"/>
+      <x:c r="J27" s="31"/>
+      <x:c r="K27" s="22"/>
+      <x:c r="L27" s="22"/>
+      <x:c r="M27" s="21"/>
+      <x:c r="N27" s="21"/>
+      <x:c r="O27" s="33"/>
+      <x:c r="P27" s="34"/>
+      <x:c r="Q27" s="35"/>
+      <x:c r="R27" s="36"/>
+      <x:c r="S27" s="35"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="29"/>
+      <x:c r="B28" s="22"/>
+      <x:c r="C28" s="21"/>
+      <x:c r="D28" s="21"/>
+      <x:c r="E28" s="21"/>
+      <x:c r="F28" s="21"/>
+      <x:c r="G28" s="21"/>
+      <x:c r="H28" s="22"/>
+      <x:c r="I28" s="21"/>
+      <x:c r="J28" s="31"/>
+      <x:c r="K28" s="22"/>
+      <x:c r="L28" s="22"/>
+      <x:c r="M28" s="21"/>
+      <x:c r="N28" s="21"/>
+      <x:c r="O28" s="33"/>
+      <x:c r="P28" s="34"/>
+      <x:c r="Q28" s="35"/>
+      <x:c r="R28" s="36"/>
+      <x:c r="S28" s="35"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="29"/>
+      <x:c r="B29" s="22"/>
+      <x:c r="C29" s="21"/>
+      <x:c r="D29" s="21"/>
+      <x:c r="E29" s="21"/>
+      <x:c r="F29" s="21"/>
+      <x:c r="G29" s="21"/>
+      <x:c r="H29" s="22"/>
+      <x:c r="I29" s="21"/>
+      <x:c r="J29" s="31"/>
+      <x:c r="K29" s="22"/>
+      <x:c r="L29" s="22"/>
+      <x:c r="M29" s="21"/>
+      <x:c r="N29" s="21"/>
+      <x:c r="O29" s="33"/>
+      <x:c r="P29" s="34"/>
+      <x:c r="Q29" s="35"/>
+      <x:c r="R29" s="36"/>
+      <x:c r="S29" s="35"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="29"/>
+      <x:c r="B30" s="22"/>
+      <x:c r="C30" s="21"/>
+      <x:c r="D30" s="21"/>
+      <x:c r="E30" s="21"/>
+      <x:c r="F30" s="21"/>
+      <x:c r="G30" s="21"/>
+      <x:c r="H30" s="22"/>
+      <x:c r="I30" s="21"/>
+      <x:c r="J30" s="31"/>
+      <x:c r="K30" s="22"/>
+      <x:c r="L30" s="22"/>
+      <x:c r="M30" s="21"/>
+      <x:c r="N30" s="21"/>
+      <x:c r="O30" s="33"/>
+      <x:c r="P30" s="34"/>
+      <x:c r="Q30" s="35"/>
+      <x:c r="R30" s="36"/>
+      <x:c r="S30" s="35"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="29"/>
+      <x:c r="B31" s="22"/>
+      <x:c r="C31" s="21"/>
+      <x:c r="D31" s="21"/>
+      <x:c r="E31" s="21"/>
+      <x:c r="F31" s="21"/>
+      <x:c r="G31" s="21"/>
+      <x:c r="H31" s="22"/>
+      <x:c r="I31" s="21"/>
+      <x:c r="J31" s="31"/>
+      <x:c r="K31" s="22"/>
+      <x:c r="L31" s="22"/>
+      <x:c r="M31" s="21"/>
+      <x:c r="N31" s="21"/>
+      <x:c r="O31" s="33"/>
+      <x:c r="P31" s="34"/>
+      <x:c r="Q31" s="35"/>
+      <x:c r="R31" s="36"/>
+      <x:c r="S31" s="35"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="29"/>
+      <x:c r="B32" s="22"/>
+      <x:c r="C32" s="21"/>
+      <x:c r="D32" s="21"/>
+      <x:c r="E32" s="21"/>
+      <x:c r="F32" s="21"/>
+      <x:c r="G32" s="21"/>
+      <x:c r="H32" s="22"/>
+      <x:c r="I32" s="21"/>
+      <x:c r="J32" s="31"/>
+      <x:c r="K32" s="22"/>
+      <x:c r="L32" s="22"/>
+      <x:c r="M32" s="21"/>
+      <x:c r="N32" s="21"/>
+      <x:c r="O32" s="33"/>
+      <x:c r="P32" s="34"/>
+      <x:c r="Q32" s="35"/>
+      <x:c r="R32" s="36"/>
+      <x:c r="S32" s="35"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="29"/>
+      <x:c r="B33" s="22"/>
+      <x:c r="C33" s="21"/>
+      <x:c r="D33" s="21"/>
+      <x:c r="E33" s="21"/>
+      <x:c r="F33" s="21"/>
+      <x:c r="G33" s="21"/>
+      <x:c r="H33" s="22"/>
+      <x:c r="I33" s="21"/>
+      <x:c r="J33" s="31"/>
+      <x:c r="K33" s="22"/>
+      <x:c r="L33" s="22"/>
+      <x:c r="M33" s="21"/>
+      <x:c r="N33" s="21"/>
+      <x:c r="O33" s="33"/>
+      <x:c r="P33" s="34"/>
+      <x:c r="Q33" s="35"/>
+      <x:c r="R33" s="36"/>
+      <x:c r="S33" s="35"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="29"/>
+      <x:c r="B34" s="22"/>
+      <x:c r="C34" s="21"/>
+      <x:c r="D34" s="21"/>
+      <x:c r="E34" s="21"/>
+      <x:c r="F34" s="21"/>
+      <x:c r="G34" s="21"/>
+      <x:c r="H34" s="22"/>
+      <x:c r="I34" s="21"/>
+      <x:c r="J34" s="31"/>
+      <x:c r="K34" s="22"/>
+      <x:c r="L34" s="22"/>
+      <x:c r="M34" s="21"/>
+      <x:c r="N34" s="21"/>
+      <x:c r="O34" s="33"/>
+      <x:c r="P34" s="34"/>
+      <x:c r="Q34" s="35"/>
+      <x:c r="R34" s="36"/>
+      <x:c r="S34" s="35"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="29"/>
+      <x:c r="B35" s="22"/>
+      <x:c r="C35" s="21"/>
+      <x:c r="D35" s="21"/>
+      <x:c r="E35" s="21"/>
+      <x:c r="F35" s="21"/>
+      <x:c r="G35" s="21"/>
+      <x:c r="H35" s="22"/>
+      <x:c r="I35" s="21"/>
+      <x:c r="J35" s="31"/>
+      <x:c r="K35" s="22"/>
+      <x:c r="L35" s="22"/>
+      <x:c r="M35" s="21"/>
+      <x:c r="N35" s="21"/>
+      <x:c r="O35" s="33"/>
+      <x:c r="P35" s="34"/>
+      <x:c r="Q35" s="35"/>
+      <x:c r="R35" s="36"/>
+      <x:c r="S35" s="35"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="29"/>
+      <x:c r="B36" s="22"/>
+      <x:c r="C36" s="21"/>
+      <x:c r="D36" s="21"/>
+      <x:c r="E36" s="21"/>
+      <x:c r="F36" s="21"/>
+      <x:c r="G36" s="21"/>
+      <x:c r="H36" s="22"/>
+      <x:c r="I36" s="21"/>
+      <x:c r="J36" s="31"/>
+      <x:c r="K36" s="22"/>
+      <x:c r="L36" s="22"/>
+      <x:c r="M36" s="21"/>
+      <x:c r="N36" s="21"/>
+      <x:c r="O36" s="33"/>
+      <x:c r="P36" s="34"/>
+      <x:c r="Q36" s="35"/>
+      <x:c r="R36" s="36"/>
+      <x:c r="S36" s="35"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="29"/>
+      <x:c r="B37" s="22"/>
+      <x:c r="C37" s="21"/>
+      <x:c r="D37" s="21"/>
+      <x:c r="E37" s="21"/>
+      <x:c r="F37" s="21"/>
+      <x:c r="G37" s="21"/>
+      <x:c r="H37" s="22"/>
+      <x:c r="I37" s="21"/>
+      <x:c r="J37" s="31"/>
+      <x:c r="K37" s="22"/>
+      <x:c r="L37" s="22"/>
+      <x:c r="M37" s="21"/>
+      <x:c r="N37" s="21"/>
+      <x:c r="O37" s="33"/>
+      <x:c r="P37" s="34"/>
+      <x:c r="Q37" s="35"/>
+      <x:c r="R37" s="36"/>
+      <x:c r="S37" s="35"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="29"/>
+      <x:c r="B38" s="22"/>
+      <x:c r="C38" s="21"/>
+      <x:c r="D38" s="21"/>
+      <x:c r="E38" s="21"/>
+      <x:c r="F38" s="21"/>
+      <x:c r="G38" s="21"/>
+      <x:c r="H38" s="22"/>
+      <x:c r="I38" s="21"/>
+      <x:c r="J38" s="31"/>
+      <x:c r="K38" s="22"/>
+      <x:c r="L38" s="22"/>
+      <x:c r="M38" s="21"/>
+      <x:c r="N38" s="21"/>
+      <x:c r="O38" s="33"/>
+      <x:c r="P38" s="34"/>
+      <x:c r="Q38" s="35"/>
+      <x:c r="R38" s="36"/>
+      <x:c r="S38" s="35"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="29"/>
+      <x:c r="B39" s="22"/>
+      <x:c r="C39" s="21"/>
+      <x:c r="D39" s="21"/>
+      <x:c r="E39" s="21"/>
+      <x:c r="F39" s="21"/>
+      <x:c r="G39" s="21"/>
+      <x:c r="H39" s="22"/>
+      <x:c r="I39" s="21"/>
+      <x:c r="J39" s="31"/>
+      <x:c r="K39" s="22"/>
+      <x:c r="L39" s="22"/>
+      <x:c r="M39" s="21"/>
+      <x:c r="N39" s="21"/>
+      <x:c r="O39" s="33"/>
+      <x:c r="P39" s="34"/>
+      <x:c r="Q39" s="35"/>
+      <x:c r="R39" s="36"/>
+      <x:c r="S39" s="35"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="29"/>
+      <x:c r="B40" s="22"/>
+      <x:c r="C40" s="21"/>
+      <x:c r="D40" s="21"/>
+      <x:c r="E40" s="21"/>
+      <x:c r="F40" s="21"/>
+      <x:c r="G40" s="21"/>
+      <x:c r="H40" s="22"/>
+      <x:c r="I40" s="21"/>
+      <x:c r="J40" s="31"/>
+      <x:c r="K40" s="22"/>
+      <x:c r="L40" s="22"/>
+      <x:c r="M40" s="21"/>
+      <x:c r="N40" s="21"/>
+      <x:c r="O40" s="33"/>
+      <x:c r="P40" s="34"/>
+      <x:c r="Q40" s="35"/>
+      <x:c r="R40" s="36"/>
+      <x:c r="S40" s="35"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="29"/>
+      <x:c r="B41" s="22"/>
+      <x:c r="C41" s="21"/>
+      <x:c r="D41" s="21"/>
+      <x:c r="E41" s="21"/>
+      <x:c r="F41" s="21"/>
+      <x:c r="G41" s="21"/>
+      <x:c r="H41" s="22"/>
+      <x:c r="I41" s="21"/>
+      <x:c r="J41" s="31"/>
+      <x:c r="K41" s="22"/>
+      <x:c r="L41" s="22"/>
+      <x:c r="M41" s="21"/>
+      <x:c r="N41" s="21"/>
+      <x:c r="O41" s="33"/>
+      <x:c r="P41" s="34"/>
+      <x:c r="Q41" s="35"/>
+      <x:c r="R41" s="36"/>
+      <x:c r="S41" s="35"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="29"/>
+      <x:c r="B42" s="22"/>
+      <x:c r="C42" s="21"/>
+      <x:c r="D42" s="21"/>
+      <x:c r="E42" s="21"/>
+      <x:c r="F42" s="21"/>
+      <x:c r="G42" s="21"/>
+      <x:c r="H42" s="22"/>
+      <x:c r="I42" s="21"/>
+      <x:c r="J42" s="31"/>
+      <x:c r="K42" s="22"/>
+      <x:c r="L42" s="22"/>
+      <x:c r="M42" s="21"/>
+      <x:c r="N42" s="21"/>
+      <x:c r="O42" s="33"/>
+      <x:c r="P42" s="34"/>
+      <x:c r="Q42" s="35"/>
+      <x:c r="R42" s="36"/>
+      <x:c r="S42" s="35"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="29"/>
+      <x:c r="B43" s="22"/>
+      <x:c r="C43" s="21"/>
+      <x:c r="D43" s="21"/>
+      <x:c r="E43" s="21"/>
+      <x:c r="F43" s="21"/>
+      <x:c r="G43" s="21"/>
+      <x:c r="H43" s="22"/>
+      <x:c r="I43" s="21"/>
+      <x:c r="J43" s="31"/>
+      <x:c r="K43" s="22"/>
+      <x:c r="L43" s="22"/>
+      <x:c r="M43" s="21"/>
+      <x:c r="N43" s="21"/>
+      <x:c r="O43" s="33"/>
+      <x:c r="P43" s="34"/>
+      <x:c r="Q43" s="35"/>
+      <x:c r="R43" s="36"/>
+      <x:c r="S43" s="35"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="29"/>
+      <x:c r="B44" s="22"/>
+      <x:c r="C44" s="21"/>
+      <x:c r="D44" s="21"/>
+      <x:c r="E44" s="21"/>
+      <x:c r="F44" s="21"/>
+      <x:c r="G44" s="21"/>
+      <x:c r="H44" s="22"/>
+      <x:c r="I44" s="21"/>
+      <x:c r="J44" s="31"/>
+      <x:c r="K44" s="22"/>
+      <x:c r="L44" s="22"/>
+      <x:c r="M44" s="21"/>
+      <x:c r="N44" s="21"/>
+      <x:c r="O44" s="33"/>
+      <x:c r="P44" s="34"/>
+      <x:c r="Q44" s="35"/>
+      <x:c r="R44" s="36"/>
+      <x:c r="S44" s="35"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="29"/>
+      <x:c r="B45" s="22"/>
+      <x:c r="C45" s="21"/>
+      <x:c r="D45" s="21"/>
+      <x:c r="E45" s="21"/>
+      <x:c r="F45" s="21"/>
+      <x:c r="G45" s="21"/>
+      <x:c r="H45" s="22"/>
+      <x:c r="I45" s="21"/>
+      <x:c r="J45" s="31"/>
+      <x:c r="K45" s="22"/>
+      <x:c r="L45" s="22"/>
+      <x:c r="M45" s="21"/>
+      <x:c r="N45" s="21"/>
+      <x:c r="O45" s="33"/>
+      <x:c r="P45" s="34"/>
+      <x:c r="Q45" s="35"/>
+      <x:c r="R45" s="36"/>
+      <x:c r="S45" s="35"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="29"/>
+      <x:c r="B46" s="22"/>
+      <x:c r="C46" s="21"/>
+      <x:c r="D46" s="21"/>
+      <x:c r="E46" s="21"/>
+      <x:c r="F46" s="21"/>
+      <x:c r="G46" s="21"/>
+      <x:c r="H46" s="22"/>
+      <x:c r="I46" s="21"/>
+      <x:c r="J46" s="31"/>
+      <x:c r="K46" s="22"/>
+      <x:c r="L46" s="22"/>
+      <x:c r="M46" s="21"/>
+      <x:c r="N46" s="21"/>
+      <x:c r="O46" s="33"/>
+      <x:c r="P46" s="34"/>
+      <x:c r="Q46" s="35"/>
+      <x:c r="R46" s="36"/>
+      <x:c r="S46" s="35"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="29"/>
+      <x:c r="B47" s="22"/>
+      <x:c r="C47" s="21"/>
+      <x:c r="D47" s="21"/>
+      <x:c r="E47" s="21"/>
+      <x:c r="F47" s="21"/>
+      <x:c r="G47" s="21"/>
+      <x:c r="H47" s="22"/>
+      <x:c r="I47" s="21"/>
+      <x:c r="J47" s="31"/>
+      <x:c r="K47" s="22"/>
+      <x:c r="L47" s="22"/>
+      <x:c r="M47" s="21"/>
+      <x:c r="N47" s="21"/>
+      <x:c r="O47" s="33"/>
+      <x:c r="P47" s="34"/>
+      <x:c r="Q47" s="35"/>
+      <x:c r="R47" s="36"/>
+      <x:c r="S47" s="35"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="29"/>
+      <x:c r="B48" s="22"/>
+      <x:c r="C48" s="21"/>
+      <x:c r="D48" s="21"/>
+      <x:c r="E48" s="21"/>
+      <x:c r="F48" s="21"/>
+      <x:c r="G48" s="21"/>
+      <x:c r="H48" s="22"/>
+      <x:c r="I48" s="21"/>
+      <x:c r="J48" s="31"/>
+      <x:c r="K48" s="22"/>
+      <x:c r="L48" s="22"/>
+      <x:c r="M48" s="21"/>
+      <x:c r="N48" s="21"/>
+      <x:c r="O48" s="33"/>
+      <x:c r="P48" s="34"/>
+      <x:c r="Q48" s="35"/>
+      <x:c r="R48" s="36"/>
+      <x:c r="S48" s="35"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="29"/>
+      <x:c r="B49" s="22"/>
+      <x:c r="C49" s="21"/>
+      <x:c r="D49" s="21"/>
+      <x:c r="E49" s="21"/>
+      <x:c r="F49" s="21"/>
+      <x:c r="G49" s="21"/>
+      <x:c r="H49" s="22"/>
+      <x:c r="I49" s="21"/>
+      <x:c r="J49" s="31"/>
+      <x:c r="K49" s="22"/>
+      <x:c r="L49" s="22"/>
+      <x:c r="M49" s="21"/>
+      <x:c r="N49" s="21"/>
+      <x:c r="O49" s="33"/>
+      <x:c r="P49" s="34"/>
+      <x:c r="Q49" s="35"/>
+      <x:c r="R49" s="36"/>
+      <x:c r="S49" s="35"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="29"/>
+      <x:c r="B50" s="22"/>
+      <x:c r="C50" s="21"/>
+      <x:c r="D50" s="21"/>
+      <x:c r="E50" s="21"/>
+      <x:c r="F50" s="21"/>
+      <x:c r="G50" s="21"/>
+      <x:c r="H50" s="22"/>
+      <x:c r="I50" s="21"/>
+      <x:c r="J50" s="31"/>
+      <x:c r="K50" s="22"/>
+      <x:c r="L50" s="22"/>
+      <x:c r="M50" s="21"/>
+      <x:c r="N50" s="21"/>
+      <x:c r="O50" s="33"/>
+      <x:c r="P50" s="34"/>
+      <x:c r="Q50" s="35"/>
+      <x:c r="R50" s="36"/>
+      <x:c r="S50" s="35"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="19"/>
+      <x:c r="B51" s="19"/>
+      <x:c r="C51" s="19"/>
+      <x:c r="D51" s="19"/>
+      <x:c r="E51" s="19"/>
+      <x:c r="F51" s="19"/>
+      <x:c r="G51" s="19"/>
+      <x:c r="H51" s="19"/>
+      <x:c r="I51" s="19"/>
+      <x:c r="J51" s="19"/>
+      <x:c r="K51" s="19"/>
+      <x:c r="L51" s="19"/>
+      <x:c r="M51" s="19"/>
+      <x:c r="N51" s="19"/>
+      <x:c r="O51" s="19"/>
+      <x:c r="P51" s="19"/>
+      <x:c r="Q51" s="19"/>
+      <x:c r="R51" s="19"/>
+      <x:c r="S51" s="19"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="19"/>
+      <x:c r="B52" s="19"/>
+      <x:c r="C52" s="19"/>
+      <x:c r="D52" s="19"/>
+      <x:c r="E52" s="19"/>
+      <x:c r="F52" s="19"/>
+      <x:c r="G52" s="19"/>
+      <x:c r="H52" s="19"/>
+      <x:c r="I52" s="19"/>
+      <x:c r="J52" s="19"/>
+      <x:c r="K52" s="19"/>
+      <x:c r="L52" s="19"/>
+      <x:c r="M52" s="19"/>
+      <x:c r="N52" s="19"/>
+      <x:c r="O52" s="19"/>
+      <x:c r="P52" s="19"/>
+      <x:c r="Q52" s="19"/>
+      <x:c r="R52" s="19"/>
+      <x:c r="S52" s="19"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="19"/>
+      <x:c r="B53" s="19"/>
+      <x:c r="C53" s="19"/>
+      <x:c r="D53" s="19"/>
+      <x:c r="E53" s="19"/>
+      <x:c r="F53" s="19"/>
+      <x:c r="G53" s="19"/>
+      <x:c r="H53" s="19"/>
+      <x:c r="I53" s="19"/>
+      <x:c r="J53" s="19"/>
+      <x:c r="K53" s="19"/>
+      <x:c r="L53" s="19"/>
+      <x:c r="M53" s="19"/>
+      <x:c r="N53" s="19"/>
+      <x:c r="O53" s="19"/>
+      <x:c r="P53" s="19"/>
+      <x:c r="Q53" s="19"/>
+      <x:c r="R53" s="19"/>
+      <x:c r="S53" s="19"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:S1"/>
+    <x:mergeCell ref="A2:S2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1167,7 +2392,7 @@
       <x:c r="G6" s="22" t="str">
         <x:v>NV-DN-01</x:v>
       </x:c>
-      <x:c r="H6" s="33" t="n">
+      <x:c r="H6" s="37" t="n">
         <x:v>46261</x:v>
       </x:c>
       <x:c r="I6" s="31" t="n">
@@ -1182,7 +2407,7 @@
       <x:c r="E7" s="32"/>
       <x:c r="F7" s="21"/>
       <x:c r="G7" s="22"/>
-      <x:c r="H7" s="33"/>
+      <x:c r="H7" s="37"/>
       <x:c r="I7" s="31"/>
     </x:row>
     <x:row r="8">
@@ -1193,7 +2418,7 @@
       <x:c r="E8" s="32"/>
       <x:c r="F8" s="21"/>
       <x:c r="G8" s="22"/>
-      <x:c r="H8" s="33"/>
+      <x:c r="H8" s="37"/>
       <x:c r="I8" s="31"/>
     </x:row>
     <x:row r="9">
@@ -1204,7 +2429,7 @@
       <x:c r="E9" s="32"/>
       <x:c r="F9" s="21"/>
       <x:c r="G9" s="22"/>
-      <x:c r="H9" s="33"/>
+      <x:c r="H9" s="37"/>
       <x:c r="I9" s="31"/>
     </x:row>
     <x:row r="10">
@@ -1215,7 +2440,7 @@
       <x:c r="E10" s="32"/>
       <x:c r="F10" s="21"/>
       <x:c r="G10" s="22"/>
-      <x:c r="H10" s="33"/>
+      <x:c r="H10" s="37"/>
       <x:c r="I10" s="31"/>
     </x:row>
     <x:row r="11">
@@ -1226,7 +2451,7 @@
       <x:c r="E11" s="32"/>
       <x:c r="F11" s="21"/>
       <x:c r="G11" s="22"/>
-      <x:c r="H11" s="33"/>
+      <x:c r="H11" s="37"/>
       <x:c r="I11" s="31"/>
     </x:row>
     <x:row r="12">
@@ -1237,7 +2462,7 @@
       <x:c r="E12" s="32"/>
       <x:c r="F12" s="21"/>
       <x:c r="G12" s="22"/>
-      <x:c r="H12" s="33"/>
+      <x:c r="H12" s="37"/>
       <x:c r="I12" s="31"/>
     </x:row>
     <x:row r="13">
@@ -1248,7 +2473,7 @@
       <x:c r="E13" s="32"/>
       <x:c r="F13" s="21"/>
       <x:c r="G13" s="22"/>
-      <x:c r="H13" s="33"/>
+      <x:c r="H13" s="37"/>
       <x:c r="I13" s="31"/>
     </x:row>
     <x:row r="14">
@@ -1259,7 +2484,7 @@
       <x:c r="E14" s="32"/>
       <x:c r="F14" s="21"/>
       <x:c r="G14" s="22"/>
-      <x:c r="H14" s="33"/>
+      <x:c r="H14" s="37"/>
       <x:c r="I14" s="31"/>
     </x:row>
     <x:row r="15">
@@ -1270,7 +2495,7 @@
       <x:c r="E15" s="32"/>
       <x:c r="F15" s="21"/>
       <x:c r="G15" s="22"/>
-      <x:c r="H15" s="33"/>
+      <x:c r="H15" s="37"/>
       <x:c r="I15" s="31"/>
     </x:row>
     <x:row r="16">
@@ -1281,7 +2506,7 @@
       <x:c r="E16" s="32"/>
       <x:c r="F16" s="21"/>
       <x:c r="G16" s="22"/>
-      <x:c r="H16" s="33"/>
+      <x:c r="H16" s="37"/>
       <x:c r="I16" s="31"/>
     </x:row>
     <x:row r="17">
@@ -1292,7 +2517,7 @@
       <x:c r="E17" s="32"/>
       <x:c r="F17" s="21"/>
       <x:c r="G17" s="22"/>
-      <x:c r="H17" s="33"/>
+      <x:c r="H17" s="37"/>
       <x:c r="I17" s="31"/>
     </x:row>
     <x:row r="18">
@@ -1303,7 +2528,7 @@
       <x:c r="E18" s="32"/>
       <x:c r="F18" s="21"/>
       <x:c r="G18" s="22"/>
-      <x:c r="H18" s="33"/>
+      <x:c r="H18" s="37"/>
       <x:c r="I18" s="31"/>
     </x:row>
     <x:row r="19">
@@ -1314,7 +2539,7 @@
       <x:c r="E19" s="32"/>
       <x:c r="F19" s="21"/>
       <x:c r="G19" s="22"/>
-      <x:c r="H19" s="33"/>
+      <x:c r="H19" s="37"/>
       <x:c r="I19" s="31"/>
     </x:row>
     <x:row r="20">
@@ -1325,7 +2550,7 @@
       <x:c r="E20" s="32"/>
       <x:c r="F20" s="21"/>
       <x:c r="G20" s="22"/>
-      <x:c r="H20" s="33"/>
+      <x:c r="H20" s="37"/>
       <x:c r="I20" s="31"/>
     </x:row>
     <x:row r="21">
@@ -1336,7 +2561,7 @@
       <x:c r="E21" s="32"/>
       <x:c r="F21" s="21"/>
       <x:c r="G21" s="22"/>
-      <x:c r="H21" s="33"/>
+      <x:c r="H21" s="37"/>
       <x:c r="I21" s="31"/>
     </x:row>
     <x:row r="22">
@@ -1347,7 +2572,7 @@
       <x:c r="E22" s="32"/>
       <x:c r="F22" s="21"/>
       <x:c r="G22" s="22"/>
-      <x:c r="H22" s="33"/>
+      <x:c r="H22" s="37"/>
       <x:c r="I22" s="31"/>
     </x:row>
     <x:row r="23">
@@ -1358,7 +2583,7 @@
       <x:c r="E23" s="32"/>
       <x:c r="F23" s="21"/>
       <x:c r="G23" s="22"/>
-      <x:c r="H23" s="33"/>
+      <x:c r="H23" s="37"/>
       <x:c r="I23" s="31"/>
     </x:row>
     <x:row r="24">
@@ -1369,7 +2594,7 @@
       <x:c r="E24" s="32"/>
       <x:c r="F24" s="21"/>
       <x:c r="G24" s="22"/>
-      <x:c r="H24" s="33"/>
+      <x:c r="H24" s="37"/>
       <x:c r="I24" s="31"/>
     </x:row>
     <x:row r="25">
@@ -1380,7 +2605,7 @@
       <x:c r="E25" s="32"/>
       <x:c r="F25" s="21"/>
       <x:c r="G25" s="22"/>
-      <x:c r="H25" s="33"/>
+      <x:c r="H25" s="37"/>
       <x:c r="I25" s="31"/>
     </x:row>
     <x:row r="26">
@@ -1391,7 +2616,7 @@
       <x:c r="E26" s="32"/>
       <x:c r="F26" s="21"/>
       <x:c r="G26" s="22"/>
-      <x:c r="H26" s="33"/>
+      <x:c r="H26" s="37"/>
       <x:c r="I26" s="31"/>
     </x:row>
     <x:row r="27">
@@ -1402,7 +2627,7 @@
       <x:c r="E27" s="32"/>
       <x:c r="F27" s="21"/>
       <x:c r="G27" s="22"/>
-      <x:c r="H27" s="33"/>
+      <x:c r="H27" s="37"/>
       <x:c r="I27" s="31"/>
     </x:row>
     <x:row r="28">
@@ -1413,7 +2638,7 @@
       <x:c r="E28" s="32"/>
       <x:c r="F28" s="21"/>
       <x:c r="G28" s="22"/>
-      <x:c r="H28" s="33"/>
+      <x:c r="H28" s="37"/>
       <x:c r="I28" s="31"/>
     </x:row>
     <x:row r="29">
@@ -1424,7 +2649,7 @@
       <x:c r="E29" s="32"/>
       <x:c r="F29" s="21"/>
       <x:c r="G29" s="22"/>
-      <x:c r="H29" s="33"/>
+      <x:c r="H29" s="37"/>
       <x:c r="I29" s="31"/>
     </x:row>
     <x:row r="30">
@@ -1435,7 +2660,7 @@
       <x:c r="E30" s="32"/>
       <x:c r="F30" s="21"/>
       <x:c r="G30" s="22"/>
-      <x:c r="H30" s="33"/>
+      <x:c r="H30" s="37"/>
       <x:c r="I30" s="31"/>
     </x:row>
     <x:row r="31">
@@ -1446,7 +2671,7 @@
       <x:c r="E31" s="32"/>
       <x:c r="F31" s="21"/>
       <x:c r="G31" s="22"/>
-      <x:c r="H31" s="33"/>
+      <x:c r="H31" s="37"/>
       <x:c r="I31" s="31"/>
     </x:row>
     <x:row r="32">
@@ -1457,7 +2682,7 @@
       <x:c r="E32" s="32"/>
       <x:c r="F32" s="21"/>
       <x:c r="G32" s="22"/>
-      <x:c r="H32" s="33"/>
+      <x:c r="H32" s="37"/>
       <x:c r="I32" s="31"/>
     </x:row>
     <x:row r="33">
@@ -1468,7 +2693,7 @@
       <x:c r="E33" s="32"/>
       <x:c r="F33" s="21"/>
       <x:c r="G33" s="22"/>
-      <x:c r="H33" s="33"/>
+      <x:c r="H33" s="37"/>
       <x:c r="I33" s="31"/>
     </x:row>
     <x:row r="34">
@@ -1479,7 +2704,7 @@
       <x:c r="E34" s="32"/>
       <x:c r="F34" s="21"/>
       <x:c r="G34" s="22"/>
-      <x:c r="H34" s="33"/>
+      <x:c r="H34" s="37"/>
       <x:c r="I34" s="31"/>
     </x:row>
     <x:row r="35">
@@ -1490,7 +2715,7 @@
       <x:c r="E35" s="32"/>
       <x:c r="F35" s="21"/>
       <x:c r="G35" s="22"/>
-      <x:c r="H35" s="33"/>
+      <x:c r="H35" s="37"/>
       <x:c r="I35" s="31"/>
     </x:row>
     <x:row r="36">
@@ -1501,7 +2726,7 @@
       <x:c r="E36" s="32"/>
       <x:c r="F36" s="21"/>
       <x:c r="G36" s="22"/>
-      <x:c r="H36" s="33"/>
+      <x:c r="H36" s="37"/>
       <x:c r="I36" s="31"/>
     </x:row>
     <x:row r="37">
@@ -1512,7 +2737,7 @@
       <x:c r="E37" s="32"/>
       <x:c r="F37" s="21"/>
       <x:c r="G37" s="22"/>
-      <x:c r="H37" s="33"/>
+      <x:c r="H37" s="37"/>
       <x:c r="I37" s="31"/>
     </x:row>
     <x:row r="38">
@@ -1523,7 +2748,7 @@
       <x:c r="E38" s="32"/>
       <x:c r="F38" s="21"/>
       <x:c r="G38" s="22"/>
-      <x:c r="H38" s="33"/>
+      <x:c r="H38" s="37"/>
       <x:c r="I38" s="31"/>
     </x:row>
     <x:row r="39">
@@ -1534,7 +2759,7 @@
       <x:c r="E39" s="32"/>
       <x:c r="F39" s="21"/>
       <x:c r="G39" s="22"/>
-      <x:c r="H39" s="33"/>
+      <x:c r="H39" s="37"/>
       <x:c r="I39" s="31"/>
     </x:row>
     <x:row r="40">
@@ -1545,7 +2770,7 @@
       <x:c r="E40" s="32"/>
       <x:c r="F40" s="21"/>
       <x:c r="G40" s="22"/>
-      <x:c r="H40" s="33"/>
+      <x:c r="H40" s="37"/>
       <x:c r="I40" s="31"/>
     </x:row>
     <x:row r="41">
@@ -1556,7 +2781,7 @@
       <x:c r="E41" s="32"/>
       <x:c r="F41" s="21"/>
       <x:c r="G41" s="22"/>
-      <x:c r="H41" s="33"/>
+      <x:c r="H41" s="37"/>
       <x:c r="I41" s="31"/>
     </x:row>
     <x:row r="42">
@@ -1567,7 +2792,7 @@
       <x:c r="E42" s="32"/>
       <x:c r="F42" s="21"/>
       <x:c r="G42" s="22"/>
-      <x:c r="H42" s="33"/>
+      <x:c r="H42" s="37"/>
       <x:c r="I42" s="31"/>
     </x:row>
     <x:row r="43">
@@ -1578,7 +2803,7 @@
       <x:c r="E43" s="32"/>
       <x:c r="F43" s="21"/>
       <x:c r="G43" s="22"/>
-      <x:c r="H43" s="33"/>
+      <x:c r="H43" s="37"/>
       <x:c r="I43" s="31"/>
     </x:row>
     <x:row r="44">
@@ -1589,7 +2814,7 @@
       <x:c r="E44" s="32"/>
       <x:c r="F44" s="21"/>
       <x:c r="G44" s="22"/>
-      <x:c r="H44" s="33"/>
+      <x:c r="H44" s="37"/>
       <x:c r="I44" s="31"/>
     </x:row>
     <x:row r="45">
@@ -1600,7 +2825,7 @@
       <x:c r="E45" s="32"/>
       <x:c r="F45" s="21"/>
       <x:c r="G45" s="22"/>
-      <x:c r="H45" s="33"/>
+      <x:c r="H45" s="37"/>
       <x:c r="I45" s="31"/>
     </x:row>
     <x:row r="46">
@@ -1611,7 +2836,7 @@
       <x:c r="E46" s="32"/>
       <x:c r="F46" s="21"/>
       <x:c r="G46" s="22"/>
-      <x:c r="H46" s="33"/>
+      <x:c r="H46" s="37"/>
       <x:c r="I46" s="31"/>
     </x:row>
     <x:row r="47">
@@ -1622,7 +2847,7 @@
       <x:c r="E47" s="32"/>
       <x:c r="F47" s="21"/>
       <x:c r="G47" s="22"/>
-      <x:c r="H47" s="33"/>
+      <x:c r="H47" s="37"/>
       <x:c r="I47" s="31"/>
     </x:row>
     <x:row r="48">
@@ -1633,7 +2858,7 @@
       <x:c r="E48" s="32"/>
       <x:c r="F48" s="21"/>
       <x:c r="G48" s="22"/>
-      <x:c r="H48" s="33"/>
+      <x:c r="H48" s="37"/>
       <x:c r="I48" s="31"/>
     </x:row>
     <x:row r="49">
@@ -1644,7 +2869,7 @@
       <x:c r="E49" s="32"/>
       <x:c r="F49" s="21"/>
       <x:c r="G49" s="22"/>
-      <x:c r="H49" s="33"/>
+      <x:c r="H49" s="37"/>
       <x:c r="I49" s="31"/>
     </x:row>
     <x:row r="50">
@@ -1655,7 +2880,7 @@
       <x:c r="E50" s="32"/>
       <x:c r="F50" s="21"/>
       <x:c r="G50" s="22"/>
-      <x:c r="H50" s="33"/>
+      <x:c r="H50" s="37"/>
       <x:c r="I50" s="31"/>
     </x:row>
     <x:row r="51">
@@ -1693,8 +2918,8 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A1:I1"/>
+    <x:mergeCell ref="A2:I2"/>
   </x:mergeCells>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="F6:F50">
@@ -1705,7 +2930,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2051,14 +3276,14 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A1:D1"/>
+    <x:mergeCell ref="A2:D2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2127,10 +3352,10 @@
       <x:c r="B6" s="22" t="str">
         <x:v>NV-DN-01</x:v>
       </x:c>
-      <x:c r="C6" s="34" t="str">
+      <x:c r="C6" s="38" t="str">
         <x:v>DB_DANANG</x:v>
       </x:c>
-      <x:c r="D6" s="34" t="str">
+      <x:c r="D6" s="38" t="str">
         <x:v>SP_NEB_3</x:v>
       </x:c>
       <x:c r="E6" s="30" t="n">
@@ -2147,10 +3372,10 @@
       <x:c r="B7" s="22" t="str">
         <x:v>NV-QN-01</x:v>
       </x:c>
-      <x:c r="C7" s="34" t="str">
+      <x:c r="C7" s="38" t="str">
         <x:v>DB_QUANGNAM</x:v>
       </x:c>
-      <x:c r="D7" s="34" t="str"/>
+      <x:c r="D7" s="38" t="str"/>
       <x:c r="E7" s="30" t="n">
         <x:v>35000000</x:v>
       </x:c>
@@ -2161,344 +3386,344 @@
     <x:row r="8">
       <x:c r="A8" s="22"/>
       <x:c r="B8" s="22"/>
-      <x:c r="C8" s="34"/>
-      <x:c r="D8" s="34"/>
+      <x:c r="C8" s="38"/>
+      <x:c r="D8" s="38"/>
       <x:c r="E8" s="30"/>
       <x:c r="F8" s="21"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="22"/>
       <x:c r="B9" s="22"/>
-      <x:c r="C9" s="34"/>
-      <x:c r="D9" s="34"/>
+      <x:c r="C9" s="38"/>
+      <x:c r="D9" s="38"/>
       <x:c r="E9" s="30"/>
       <x:c r="F9" s="21"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="22"/>
       <x:c r="B10" s="22"/>
-      <x:c r="C10" s="34"/>
-      <x:c r="D10" s="34"/>
+      <x:c r="C10" s="38"/>
+      <x:c r="D10" s="38"/>
       <x:c r="E10" s="30"/>
       <x:c r="F10" s="21"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="22"/>
       <x:c r="B11" s="22"/>
-      <x:c r="C11" s="34"/>
-      <x:c r="D11" s="34"/>
+      <x:c r="C11" s="38"/>
+      <x:c r="D11" s="38"/>
       <x:c r="E11" s="30"/>
       <x:c r="F11" s="21"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="22"/>
       <x:c r="B12" s="22"/>
-      <x:c r="C12" s="34"/>
-      <x:c r="D12" s="34"/>
+      <x:c r="C12" s="38"/>
+      <x:c r="D12" s="38"/>
       <x:c r="E12" s="30"/>
       <x:c r="F12" s="21"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="22"/>
       <x:c r="B13" s="22"/>
-      <x:c r="C13" s="34"/>
-      <x:c r="D13" s="34"/>
+      <x:c r="C13" s="38"/>
+      <x:c r="D13" s="38"/>
       <x:c r="E13" s="30"/>
       <x:c r="F13" s="21"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="22"/>
       <x:c r="B14" s="22"/>
-      <x:c r="C14" s="34"/>
-      <x:c r="D14" s="34"/>
+      <x:c r="C14" s="38"/>
+      <x:c r="D14" s="38"/>
       <x:c r="E14" s="30"/>
       <x:c r="F14" s="21"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="22"/>
       <x:c r="B15" s="22"/>
-      <x:c r="C15" s="34"/>
-      <x:c r="D15" s="34"/>
+      <x:c r="C15" s="38"/>
+      <x:c r="D15" s="38"/>
       <x:c r="E15" s="30"/>
       <x:c r="F15" s="21"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="22"/>
       <x:c r="B16" s="22"/>
-      <x:c r="C16" s="34"/>
-      <x:c r="D16" s="34"/>
+      <x:c r="C16" s="38"/>
+      <x:c r="D16" s="38"/>
       <x:c r="E16" s="30"/>
       <x:c r="F16" s="21"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="22"/>
       <x:c r="B17" s="22"/>
-      <x:c r="C17" s="34"/>
-      <x:c r="D17" s="34"/>
+      <x:c r="C17" s="38"/>
+      <x:c r="D17" s="38"/>
       <x:c r="E17" s="30"/>
       <x:c r="F17" s="21"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="22"/>
       <x:c r="B18" s="22"/>
-      <x:c r="C18" s="34"/>
-      <x:c r="D18" s="34"/>
+      <x:c r="C18" s="38"/>
+      <x:c r="D18" s="38"/>
       <x:c r="E18" s="30"/>
       <x:c r="F18" s="21"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="22"/>
       <x:c r="B19" s="22"/>
-      <x:c r="C19" s="34"/>
-      <x:c r="D19" s="34"/>
+      <x:c r="C19" s="38"/>
+      <x:c r="D19" s="38"/>
       <x:c r="E19" s="30"/>
       <x:c r="F19" s="21"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="22"/>
       <x:c r="B20" s="22"/>
-      <x:c r="C20" s="34"/>
-      <x:c r="D20" s="34"/>
+      <x:c r="C20" s="38"/>
+      <x:c r="D20" s="38"/>
       <x:c r="E20" s="30"/>
       <x:c r="F20" s="21"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="22"/>
       <x:c r="B21" s="22"/>
-      <x:c r="C21" s="34"/>
-      <x:c r="D21" s="34"/>
+      <x:c r="C21" s="38"/>
+      <x:c r="D21" s="38"/>
       <x:c r="E21" s="30"/>
       <x:c r="F21" s="21"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="22"/>
       <x:c r="B22" s="22"/>
-      <x:c r="C22" s="34"/>
-      <x:c r="D22" s="34"/>
+      <x:c r="C22" s="38"/>
+      <x:c r="D22" s="38"/>
       <x:c r="E22" s="30"/>
       <x:c r="F22" s="21"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="22"/>
       <x:c r="B23" s="22"/>
-      <x:c r="C23" s="34"/>
-      <x:c r="D23" s="34"/>
+      <x:c r="C23" s="38"/>
+      <x:c r="D23" s="38"/>
       <x:c r="E23" s="30"/>
       <x:c r="F23" s="21"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="22"/>
       <x:c r="B24" s="22"/>
-      <x:c r="C24" s="34"/>
-      <x:c r="D24" s="34"/>
+      <x:c r="C24" s="38"/>
+      <x:c r="D24" s="38"/>
       <x:c r="E24" s="30"/>
       <x:c r="F24" s="21"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="22"/>
       <x:c r="B25" s="22"/>
-      <x:c r="C25" s="34"/>
-      <x:c r="D25" s="34"/>
+      <x:c r="C25" s="38"/>
+      <x:c r="D25" s="38"/>
       <x:c r="E25" s="30"/>
       <x:c r="F25" s="21"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="22"/>
       <x:c r="B26" s="22"/>
-      <x:c r="C26" s="34"/>
-      <x:c r="D26" s="34"/>
+      <x:c r="C26" s="38"/>
+      <x:c r="D26" s="38"/>
       <x:c r="E26" s="30"/>
       <x:c r="F26" s="21"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="22"/>
       <x:c r="B27" s="22"/>
-      <x:c r="C27" s="34"/>
-      <x:c r="D27" s="34"/>
+      <x:c r="C27" s="38"/>
+      <x:c r="D27" s="38"/>
       <x:c r="E27" s="30"/>
       <x:c r="F27" s="21"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="22"/>
       <x:c r="B28" s="22"/>
-      <x:c r="C28" s="34"/>
-      <x:c r="D28" s="34"/>
+      <x:c r="C28" s="38"/>
+      <x:c r="D28" s="38"/>
       <x:c r="E28" s="30"/>
       <x:c r="F28" s="21"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="22"/>
       <x:c r="B29" s="22"/>
-      <x:c r="C29" s="34"/>
-      <x:c r="D29" s="34"/>
+      <x:c r="C29" s="38"/>
+      <x:c r="D29" s="38"/>
       <x:c r="E29" s="30"/>
       <x:c r="F29" s="21"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="22"/>
       <x:c r="B30" s="22"/>
-      <x:c r="C30" s="34"/>
-      <x:c r="D30" s="34"/>
+      <x:c r="C30" s="38"/>
+      <x:c r="D30" s="38"/>
       <x:c r="E30" s="30"/>
       <x:c r="F30" s="21"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="22"/>
       <x:c r="B31" s="22"/>
-      <x:c r="C31" s="34"/>
-      <x:c r="D31" s="34"/>
+      <x:c r="C31" s="38"/>
+      <x:c r="D31" s="38"/>
       <x:c r="E31" s="30"/>
       <x:c r="F31" s="21"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="22"/>
       <x:c r="B32" s="22"/>
-      <x:c r="C32" s="34"/>
-      <x:c r="D32" s="34"/>
+      <x:c r="C32" s="38"/>
+      <x:c r="D32" s="38"/>
       <x:c r="E32" s="30"/>
       <x:c r="F32" s="21"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="22"/>
       <x:c r="B33" s="22"/>
-      <x:c r="C33" s="34"/>
-      <x:c r="D33" s="34"/>
+      <x:c r="C33" s="38"/>
+      <x:c r="D33" s="38"/>
       <x:c r="E33" s="30"/>
       <x:c r="F33" s="21"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="22"/>
       <x:c r="B34" s="22"/>
-      <x:c r="C34" s="34"/>
-      <x:c r="D34" s="34"/>
+      <x:c r="C34" s="38"/>
+      <x:c r="D34" s="38"/>
       <x:c r="E34" s="30"/>
       <x:c r="F34" s="21"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="22"/>
       <x:c r="B35" s="22"/>
-      <x:c r="C35" s="34"/>
-      <x:c r="D35" s="34"/>
+      <x:c r="C35" s="38"/>
+      <x:c r="D35" s="38"/>
       <x:c r="E35" s="30"/>
       <x:c r="F35" s="21"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="22"/>
       <x:c r="B36" s="22"/>
-      <x:c r="C36" s="34"/>
-      <x:c r="D36" s="34"/>
+      <x:c r="C36" s="38"/>
+      <x:c r="D36" s="38"/>
       <x:c r="E36" s="30"/>
       <x:c r="F36" s="21"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="22"/>
       <x:c r="B37" s="22"/>
-      <x:c r="C37" s="34"/>
-      <x:c r="D37" s="34"/>
+      <x:c r="C37" s="38"/>
+      <x:c r="D37" s="38"/>
       <x:c r="E37" s="30"/>
       <x:c r="F37" s="21"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="22"/>
       <x:c r="B38" s="22"/>
-      <x:c r="C38" s="34"/>
-      <x:c r="D38" s="34"/>
+      <x:c r="C38" s="38"/>
+      <x:c r="D38" s="38"/>
       <x:c r="E38" s="30"/>
       <x:c r="F38" s="21"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="22"/>
       <x:c r="B39" s="22"/>
-      <x:c r="C39" s="34"/>
-      <x:c r="D39" s="34"/>
+      <x:c r="C39" s="38"/>
+      <x:c r="D39" s="38"/>
       <x:c r="E39" s="30"/>
       <x:c r="F39" s="21"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="22"/>
       <x:c r="B40" s="22"/>
-      <x:c r="C40" s="34"/>
-      <x:c r="D40" s="34"/>
+      <x:c r="C40" s="38"/>
+      <x:c r="D40" s="38"/>
       <x:c r="E40" s="30"/>
       <x:c r="F40" s="21"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="22"/>
       <x:c r="B41" s="22"/>
-      <x:c r="C41" s="34"/>
-      <x:c r="D41" s="34"/>
+      <x:c r="C41" s="38"/>
+      <x:c r="D41" s="38"/>
       <x:c r="E41" s="30"/>
       <x:c r="F41" s="21"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="22"/>
       <x:c r="B42" s="22"/>
-      <x:c r="C42" s="34"/>
-      <x:c r="D42" s="34"/>
+      <x:c r="C42" s="38"/>
+      <x:c r="D42" s="38"/>
       <x:c r="E42" s="30"/>
       <x:c r="F42" s="21"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="22"/>
       <x:c r="B43" s="22"/>
-      <x:c r="C43" s="34"/>
-      <x:c r="D43" s="34"/>
+      <x:c r="C43" s="38"/>
+      <x:c r="D43" s="38"/>
       <x:c r="E43" s="30"/>
       <x:c r="F43" s="21"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="22"/>
       <x:c r="B44" s="22"/>
-      <x:c r="C44" s="34"/>
-      <x:c r="D44" s="34"/>
+      <x:c r="C44" s="38"/>
+      <x:c r="D44" s="38"/>
       <x:c r="E44" s="30"/>
       <x:c r="F44" s="21"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="22"/>
       <x:c r="B45" s="22"/>
-      <x:c r="C45" s="34"/>
-      <x:c r="D45" s="34"/>
+      <x:c r="C45" s="38"/>
+      <x:c r="D45" s="38"/>
       <x:c r="E45" s="30"/>
       <x:c r="F45" s="21"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="22"/>
       <x:c r="B46" s="22"/>
-      <x:c r="C46" s="34"/>
-      <x:c r="D46" s="34"/>
+      <x:c r="C46" s="38"/>
+      <x:c r="D46" s="38"/>
       <x:c r="E46" s="30"/>
       <x:c r="F46" s="21"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="22"/>
       <x:c r="B47" s="22"/>
-      <x:c r="C47" s="34"/>
-      <x:c r="D47" s="34"/>
+      <x:c r="C47" s="38"/>
+      <x:c r="D47" s="38"/>
       <x:c r="E47" s="30"/>
       <x:c r="F47" s="21"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="22"/>
       <x:c r="B48" s="22"/>
-      <x:c r="C48" s="34"/>
-      <x:c r="D48" s="34"/>
+      <x:c r="C48" s="38"/>
+      <x:c r="D48" s="38"/>
       <x:c r="E48" s="30"/>
       <x:c r="F48" s="21"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="22"/>
       <x:c r="B49" s="22"/>
-      <x:c r="C49" s="34"/>
-      <x:c r="D49" s="34"/>
+      <x:c r="C49" s="38"/>
+      <x:c r="D49" s="38"/>
       <x:c r="E49" s="30"/>
       <x:c r="F49" s="21"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="22"/>
       <x:c r="B50" s="22"/>
-      <x:c r="C50" s="34"/>
-      <x:c r="D50" s="34"/>
+      <x:c r="C50" s="38"/>
+      <x:c r="D50" s="38"/>
       <x:c r="E50" s="30"/>
       <x:c r="F50" s="21"/>
     </x:row>
@@ -2528,8 +3753,8 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3034,8 +4259,8 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A1:C1"/>
+    <x:mergeCell ref="A2:C2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3454,8 +4679,8 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A1:E1"/>
+    <x:mergeCell ref="A2:E2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="D6:D50">
@@ -3770,8 +4995,8 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A1:C1"/>
+    <x:mergeCell ref="A2:C2"/>
   </x:mergeCells>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="C6:C50">
@@ -4914,8 +6139,8 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="C6:C50">
@@ -5165,8 +6390,8 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A1:B1"/>
+    <x:mergeCell ref="A2:B2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5644,8 +6869,8 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>